<commit_message>
Revalidación del 11-10-2026 con GLM-5.3-Flash y el modelo gratuito de opencode
- validacion.json: 38 de 38 con GLM (F.3 y EJ 21 en modo interactivo; F.0 y F.1 como programas) y 33 de 33 de los
  ejercicios con encargo también con el modelo gratuito (big-pickle). Notas nuevas de lo que pasó en los que cambiaron.
- Soluciones reales regeneradas (incluidas F.3 y EJ 21 en interactivo), anonimizadas.
- Enunciados y soluciones dicen también el resultado con el modelo gratuito.
- Presentación y PDF con los datos nuevos; README con validación y coste al día.
- Wiki de modelos: el límite de uso es por modelo y qué hacer si se agota.
</commit_message>
<xml_diff>
--- a/alumnos/soluciones/ej18_facturas_excel/ficheros/facturas.xlsx
+++ b/alumnos/soluciones/ej18_facturas_excel/ficheros/facturas.xlsx
@@ -16,7 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00 &quot;EUR&quot;"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -49,12 +53,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,15 +427,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,27 +445,22 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nº factura</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Base imponible</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Base imponible (EUR)</t>
+          <t>IVA</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>IVA 21% (EUR)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total (EUR)</t>
+          <t>Total</t>
         </is>
       </c>
     </row>
@@ -469,23 +470,16 @@
           <t>Ferretería Etxeberria</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026/041</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>03/02/2026</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="B2" s="2" t="n">
+        <v>46056</v>
+      </c>
+      <c r="C2" s="3" t="n">
         <v>375.6</v>
       </c>
-      <c r="E2" t="n">
+      <c r="D2" s="3" t="n">
         <v>78.88</v>
       </c>
-      <c r="F2" t="n">
+      <c r="E2" s="3" t="n">
         <v>454.48</v>
       </c>
     </row>
@@ -495,41 +489,29 @@
           <t>Limpiezas Ribera S.L.</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026/019</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>28/02/2026</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="B3" s="2" t="n">
+        <v>46081</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>1002.4</v>
       </c>
-      <c r="E3" t="n">
+      <c r="D3" s="3" t="n">
         <v>210.5</v>
       </c>
-      <c r="F3" t="n">
+      <c r="E3" s="3" t="n">
         <v>1212.9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>SUMA</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="n">
-        <v>1378</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>289.38</v>
-      </c>
-      <c r="F4" s="2" t="n">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>SUMA TOTAL</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="5" t="n">
         <v>1667.38</v>
       </c>
     </row>

</xml_diff>